<commit_message>
VFE template - updated to jxls3
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/teams/VFE_Teams-A4.xlsx
+++ b/owlcms/src/main/resources/templates/teams/VFE_Teams-A4.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\git\owlcms4\owlcms\src\main\resources\templates\teams\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A84B9889-3FDD-4A92-ABE6-B31D6032E8C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBDAE707-CD3C-434A-81CB-E2FD1815BE20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6000" yWindow="3300" windowWidth="22410" windowHeight="15555" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6345" yWindow="3645" windowWidth="22410" windowHeight="15555" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Team List" sheetId="3" r:id="rId1"/>
@@ -545,6 +545,9 @@
     <xf numFmtId="1" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
@@ -557,9 +560,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1007,16 +1007,16 @@
       <c r="B2" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="45" t="s">
+      <c r="C2" s="46" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
-      <c r="H2" s="45"/>
-      <c r="I2" s="45"/>
-      <c r="J2" s="45"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="46"/>
+      <c r="I2" s="46"/>
+      <c r="J2" s="46"/>
       <c r="L2" s="4"/>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
@@ -1037,14 +1037,14 @@
         <v>4</v>
       </c>
       <c r="D3" s="6"/>
-      <c r="E3" s="46" t="s">
+      <c r="E3" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
-      <c r="H3" s="46"/>
-      <c r="I3" s="46"/>
-      <c r="J3" s="46"/>
+      <c r="F3" s="47"/>
+      <c r="G3" s="47"/>
+      <c r="H3" s="47"/>
+      <c r="I3" s="47"/>
+      <c r="J3" s="47"/>
       <c r="L3" s="4"/>
       <c r="N3" s="1"/>
       <c r="O3" s="1"/>
@@ -1065,14 +1065,14 @@
         <v>7</v>
       </c>
       <c r="D4" s="8"/>
-      <c r="E4" s="48" t="s">
+      <c r="E4" s="49" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="48"/>
-      <c r="G4" s="48"/>
-      <c r="H4" s="48"/>
-      <c r="I4" s="48"/>
-      <c r="J4" s="48"/>
+      <c r="F4" s="49"/>
+      <c r="G4" s="49"/>
+      <c r="H4" s="49"/>
+      <c r="I4" s="49"/>
+      <c r="J4" s="49"/>
       <c r="L4" s="4"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
@@ -1083,18 +1083,18 @@
       <c r="X4"/>
     </row>
     <row r="5" spans="1:24" s="9" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="49" t="s">
+      <c r="A5" s="45" t="s">
         <v>28</v>
       </c>
-      <c r="B5" s="49"/>
-      <c r="C5" s="49"/>
-      <c r="D5" s="49"/>
-      <c r="E5" s="49"/>
-      <c r="F5" s="49"/>
-      <c r="G5" s="49"/>
-      <c r="H5" s="49"/>
-      <c r="I5" s="49"/>
-      <c r="J5" s="49"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="45"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="45"/>
+      <c r="I5" s="45"/>
+      <c r="J5" s="45"/>
       <c r="K5" s="10"/>
       <c r="L5" s="11"/>
       <c r="M5" s="12"/>
@@ -1331,11 +1331,11 @@
       <c r="M15" s="19"/>
     </row>
     <row r="16" spans="1:24" s="20" customFormat="1" ht="62.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="47" t="s">
+      <c r="A16" s="48" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="47"/>
-      <c r="C16" s="47"/>
+      <c r="B16" s="48"/>
+      <c r="C16" s="48"/>
       <c r="D16" s="35"/>
       <c r="E16" s="36"/>
       <c r="F16" s="17"/>
@@ -2615,12 +2615,11 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
-  <mergeCells count="5">
+  <mergeCells count="4">
     <mergeCell ref="C2:J2"/>
     <mergeCell ref="E3:J3"/>
     <mergeCell ref="A16:C16"/>
     <mergeCell ref="E4:J4"/>
-    <mergeCell ref="A5:J5"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="decimal" allowBlank="1" showErrorMessage="1" sqref="K10 K6 K11:K12" xr:uid="{00000000-0002-0000-0000-000000000000}">

</xml_diff>